<commit_message>
docs(comms): add Onboarding Tour tab - localhost-only verify for HP
Arrow-pointer + drag polish on the new-player tour, held uncommitted
pending Xero's look. Not blocking.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tasks/The Tapestry Smoke Testing.xlsx
+++ b/tasks/The Tapestry Smoke Testing.xlsx
@@ -11,6 +11,7 @@
     <sheet name="New Fixes 2026-07-13" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Mechanics Verify 2026-07-06" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Portrait Bank 2026-08-03" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Onboarding Tour 2026-08-04" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Full Smoke 2026-07-13'!$A$1:$E$58</definedName>
@@ -789,50 +790,64 @@
       </c>
     </row>
     <row r="11" ht="15.75" customHeight="1" s="31">
-      <c r="B11" s="8" t="inlineStr">
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Onboarding Tour 2026-08-04</t>
+        </is>
+      </c>
+      <c r="C11" s="42" t="inlineStr">
+        <is>
+          <t>5 items</t>
+        </is>
+      </c>
+      <c r="D11" s="41" t="inlineStr">
+        <is>
+          <t>None run yet. LOCALHOST ONLY (dev server). Arrow-pointer + drag polish on the new-player tour, held uncommitted pending your look.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="27.95" customHeight="1" s="31">
+      <c r="B12" s="43" t="inlineStr">
         <is>
           <t>FASTEST PATH</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="27.95" customHeight="1" s="31">
-      <c r="B12" s="30" t="inlineStr">
-        <is>
-          <t>1. Full Smoke tab: the 9 open items sit at the TOP (amber = quick confirm, red = real unknown). Everything below the grey divider already passed - ignore it.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="27.95" customHeight="1" s="31">
       <c r="B13" s="30" t="inlineStr">
         <is>
-          <t>2. New Fixes + Mechanics tabs: every row needs you; work top to bottom.</t>
+          <t>1. Full Smoke tab: the 9 open items sit at the TOP (amber = quick confirm, red = real unknown). Everything below the grey divider already passed - ignore it.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="27.95" customHeight="1" s="31">
       <c r="B14" s="30" t="inlineStr">
         <is>
-          <t>3. Mark the Result column (dropdown) as you go. Amber/red/blue rows = action; grey rows = done.</t>
+          <t>2. New Fixes + Mechanics tabs: every row needs you; work top to bottom.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="27.95" customHeight="1" s="31">
       <c r="B15" s="30" t="inlineStr">
         <is>
+          <t>3. Mark the Result column (dropdown) as you go. Amber/red/blue rows = action; grey rows = done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="41" t="inlineStr">
+        <is>
           <t>4. Tip: click the filter arrow on 'Status' to show only what you want (e.g. hide DONE).</t>
         </is>
       </c>
-    </row>
-    <row r="16">
-      <c r="B16" s="41" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="B14:D14"/>
-    <mergeCell ref="B15:D15"/>
     <mergeCell ref="B4:D4"/>
     <mergeCell ref="B13:D13"/>
-    <mergeCell ref="B12:D12"/>
+    <mergeCell ref="B15:D15"/>
+    <mergeCell ref="B16:D16"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3398,4 +3413,183 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="7" customWidth="1" style="31" min="1" max="1"/>
+    <col width="15" customWidth="1" style="31" min="2" max="2"/>
+    <col width="100" customWidth="1" style="31" min="3" max="3"/>
+    <col width="30" customWidth="1" style="31" min="4" max="4"/>
+    <col width="46" customWidth="1" style="31" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="33" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B1" s="33" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="C1" s="33" t="inlineStr">
+        <is>
+          <t>Do this</t>
+        </is>
+      </c>
+      <c r="D1" s="33" t="inlineStr">
+        <is>
+          <t>What you saw</t>
+        </is>
+      </c>
+      <c r="E1" s="33" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="38" customHeight="1" s="31">
+      <c r="A2" s="34" t="n"/>
+      <c r="B2" s="34" t="n"/>
+      <c r="C2" s="35" t="inlineStr">
+        <is>
+          <t>READ FIRST - this is localhost only (dev server, not live). Hunt &amp; Peck is holding these changes uncommitted until you've seen them - nothing ships until you weigh in. Make sure the dev server is running (Start-Tapestry.bat), then work top to bottom.</t>
+        </is>
+      </c>
+      <c r="D2" s="34" t="n"/>
+      <c r="E2" s="34" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="36" t="n"/>
+      <c r="B3" s="36" t="n"/>
+      <c r="C3" s="37" t="inlineStr">
+        <is>
+          <t>Onboarding tour - arrow pointer + drag</t>
+        </is>
+      </c>
+      <c r="D3" s="36" t="n"/>
+      <c r="E3" s="36" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="38" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B4" s="39" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="C4" s="38" t="inlineStr">
+        <is>
+          <t>Go to localhost:3000/welcome. The tour opens automatically.</t>
+        </is>
+      </c>
+      <c r="D4" s="38" t="n"/>
+      <c r="E4" s="40" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="38" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B5" s="39" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="C5" s="38" t="inlineStr">
+        <is>
+          <t>Click Next through all 6 steps.</t>
+        </is>
+      </c>
+      <c r="D5" s="38" t="n"/>
+      <c r="E5" s="40" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="38" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B6" s="39" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="C6" s="38" t="inlineStr">
+        <is>
+          <t>On steps 2-5, watch the left sidebar: a red ring + arrow should point at a link - step 2 = the Tapestry logo, 3 = My Survivors, 4 = The Campfire, 5 = The World. Steps 1 and 6 have no arrow (by design).</t>
+        </is>
+      </c>
+      <c r="D6" s="38" t="n"/>
+      <c r="E6" s="40" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="38" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B7" s="39" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="C7" s="38" t="inlineStr">
+        <is>
+          <t>Grab the modal by the three-dot grip strip at its very top and drag it around the screen.</t>
+        </is>
+      </c>
+      <c r="D7" s="38" t="n"/>
+      <c r="E7" s="40" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="38" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B8" s="39" t="inlineStr">
+        <is>
+          <t>REPORT</t>
+        </is>
+      </c>
+      <c r="C8" s="38" t="inlineStr">
+        <is>
+          <t>Do the arrows point at the right things? Does the drag feel right? Is the backdrop dimness (a light scrim, not a blackout) about right? Does pointing at the logo for the "Dashboard" step read OK, or should that step drop its arrow?</t>
+        </is>
+      </c>
+      <c r="D8" s="38" t="n"/>
+      <c r="E8" s="40" t="n"/>
+    </row>
+    <row r="10">
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>Report back</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="C11" s="41" t="inlineStr">
+        <is>
+          <t>Fill in "What you saw" for row 5 (free text, no pass/fail needed) and send it back. HP commits + pushes once you've signed off.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>